<commit_message>
SPM-57: Record Kristen's test case run (9 pass) and refresh the matrix
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/test-cases/SPM-57_Test_Cases.xlsx
+++ b/docs/test-cases/SPM-57_Test_Cases.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\IS212\docs\test-cases\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\krist\Documents\GitHub\IS212\docs\test-cases\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EFCB3881-3CE9-4A64-8E1C-7799D8F930F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{41855CB1-C60E-475B-833A-BD5D9069E32E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="11625" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="12336" firstSheet="6" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Summary" sheetId="1" r:id="rId1"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="337" uniqueCount="127">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="445" uniqueCount="129">
   <si>
     <t>Story</t>
   </si>
@@ -505,6 +505,12 @@
   </si>
   <si>
     <t>Step 1: As Priya Raj the event opened with no 'Attendees' tab. Step 3: Typing /events/&lt;reference&gt;/attendees showed 'Not authorised' and 'You can only view the registrations for events you are responsible for.', with no 'Add attendee' button.</t>
+  </si>
+  <si>
+    <t>70a12f9</t>
+  </si>
+  <si>
+    <t>Kristen</t>
   </si>
 </sst>
 </file>
@@ -905,7 +911,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:I22"/>
-  <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="20" customWidth="1"/>
@@ -918,7 +924,7 @@
     <col min="9" max="9" width="16" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="31.05" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:9" ht="31.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="7" t="s">
         <v>0</v>
       </c>
@@ -933,7 +939,7 @@
       <c r="H1" s="17"/>
       <c r="I1" s="18"/>
     </row>
-    <row r="3" spans="1:9" ht="13.15" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" s="7" t="s">
         <v>2</v>
       </c>
@@ -962,7 +968,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:9" ht="38.25" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:9" ht="39.6" x14ac:dyDescent="0.25">
       <c r="A4" s="8" t="s">
         <v>11</v>
       </c>
@@ -987,7 +993,7 @@
       <c r="H4" s="9"/>
       <c r="I4" s="9"/>
     </row>
-    <row r="5" spans="1:9" ht="38.25" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:9" ht="39.6" x14ac:dyDescent="0.25">
       <c r="A5" s="8" t="s">
         <v>18</v>
       </c>
@@ -1012,7 +1018,7 @@
       <c r="H5" s="9"/>
       <c r="I5" s="9"/>
     </row>
-    <row r="6" spans="1:9" ht="25.5" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:9" ht="26.4" x14ac:dyDescent="0.25">
       <c r="A6" s="8" t="s">
         <v>22</v>
       </c>
@@ -1037,7 +1043,7 @@
       <c r="H6" s="9"/>
       <c r="I6" s="9"/>
     </row>
-    <row r="7" spans="1:9" ht="25.5" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:9" ht="26.4" x14ac:dyDescent="0.25">
       <c r="A7" s="8" t="s">
         <v>26</v>
       </c>
@@ -1062,7 +1068,7 @@
       <c r="H7" s="9"/>
       <c r="I7" s="9"/>
     </row>
-    <row r="8" spans="1:9" ht="25.5" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:9" ht="26.4" x14ac:dyDescent="0.25">
       <c r="A8" s="8" t="s">
         <v>31</v>
       </c>
@@ -1087,7 +1093,7 @@
       <c r="H8" s="9"/>
       <c r="I8" s="9"/>
     </row>
-    <row r="9" spans="1:9" ht="38.25" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:9" ht="39.6" x14ac:dyDescent="0.25">
       <c r="A9" s="8" t="s">
         <v>34</v>
       </c>
@@ -1112,7 +1118,7 @@
       <c r="H9" s="9"/>
       <c r="I9" s="9"/>
     </row>
-    <row r="10" spans="1:9" ht="25.5" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:9" ht="26.4" x14ac:dyDescent="0.25">
       <c r="A10" s="8" t="s">
         <v>38</v>
       </c>
@@ -1137,7 +1143,7 @@
       <c r="H10" s="9"/>
       <c r="I10" s="9"/>
     </row>
-    <row r="11" spans="1:9" ht="25.5" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:9" ht="26.4" x14ac:dyDescent="0.25">
       <c r="A11" s="8" t="s">
         <v>43</v>
       </c>
@@ -1162,7 +1168,7 @@
       <c r="H11" s="9"/>
       <c r="I11" s="9"/>
     </row>
-    <row r="12" spans="1:9" ht="25.5" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:9" ht="26.4" x14ac:dyDescent="0.25">
       <c r="A12" s="8" t="s">
         <v>46</v>
       </c>
@@ -1187,7 +1193,7 @@
       <c r="H12" s="9"/>
       <c r="I12" s="9"/>
     </row>
-    <row r="15" spans="1:9" ht="13.15" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A15" s="7" t="s">
         <v>49</v>
       </c>
@@ -1201,7 +1207,7 @@
       </c>
       <c r="F15" s="18"/>
     </row>
-    <row r="16" spans="1:9" ht="98.55" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:9" ht="98.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="9" t="s">
         <v>29</v>
       </c>
@@ -1215,7 +1221,7 @@
       </c>
       <c r="F16" s="18"/>
     </row>
-    <row r="17" spans="1:9" ht="31.05" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:9" ht="31.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="9" t="s">
         <v>54</v>
       </c>
@@ -1229,7 +1235,7 @@
       </c>
       <c r="F17" s="18"/>
     </row>
-    <row r="18" spans="1:9" ht="71.55" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:9" ht="71.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="9" t="s">
         <v>57</v>
       </c>
@@ -1243,7 +1249,7 @@
       </c>
       <c r="F18" s="18"/>
     </row>
-    <row r="19" spans="1:9" ht="31.05" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:9" ht="31.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="9" t="s">
         <v>21</v>
       </c>
@@ -1257,7 +1263,7 @@
       </c>
       <c r="F19" s="18"/>
     </row>
-    <row r="20" spans="1:9" ht="17.55" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:9" ht="17.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="9" t="s">
         <v>61</v>
       </c>
@@ -1271,7 +1277,7 @@
       </c>
       <c r="F20" s="18"/>
     </row>
-    <row r="22" spans="1:9" ht="206.55" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:9" ht="206.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="7" t="s">
         <v>63</v>
       </c>
@@ -1323,20 +1329,20 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:C17"/>
-  <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:C25"/>
+  <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="24.796875" customWidth="1"/>
-    <col min="2" max="2" width="56.796875" customWidth="1"/>
+    <col min="1" max="1" width="24.77734375" customWidth="1"/>
+    <col min="2" max="2" width="56.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="13.15" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>65</v>
       </c>
       <c r="B1" s="2"/>
     </row>
-    <row r="2" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="10" t="s">
         <v>3</v>
       </c>
@@ -1344,7 +1350,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="31.05" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:3" ht="31.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="10" t="s">
         <v>66</v>
       </c>
@@ -1352,7 +1358,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="71.55" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:3" ht="71.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="10" t="s">
         <v>67</v>
       </c>
@@ -1360,7 +1366,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="85.05" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:3" ht="85.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="10" t="s">
         <v>69</v>
       </c>
@@ -1368,7 +1374,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="31.05" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:3" ht="31.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="10" t="s">
         <v>71</v>
       </c>
@@ -1376,7 +1382,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="58.05" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:3" ht="58.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="10" t="s">
         <v>73</v>
       </c>
@@ -1384,7 +1390,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="10" t="s">
         <v>75</v>
       </c>
@@ -1392,7 +1398,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="12.75" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A9" s="10" t="s">
         <v>77</v>
       </c>
@@ -1400,15 +1406,15 @@
         <v>46323</v>
       </c>
     </row>
-    <row r="10" spans="1:3" ht="12.75" x14ac:dyDescent="0.35"/>
-    <row r="11" spans="1:3" ht="13.15" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:3" ht="13.2" x14ac:dyDescent="0.25"/>
+    <row r="11" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
         <v>65</v>
       </c>
       <c r="B11" s="5"/>
       <c r="C11" s="6"/>
     </row>
-    <row r="12" spans="1:3" ht="71.55" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:3" ht="71.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
         <v>78</v>
       </c>
@@ -1416,7 +1422,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="13" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
         <v>80</v>
       </c>
@@ -1424,7 +1430,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="14" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
         <v>82</v>
       </c>
@@ -1432,7 +1438,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="15" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
         <v>84</v>
       </c>
@@ -1440,7 +1446,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="16" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
         <v>85</v>
       </c>
@@ -1448,15 +1454,65 @@
         <v>46323</v>
       </c>
     </row>
-    <row r="17" spans="1:2" ht="17.55" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:2" ht="17.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
         <v>86</v>
       </c>
-      <c r="B17" s="13" t="inlineStr">
-        <is>
-          <t>70a12f9</t>
-        </is>
-      </c>
+      <c r="B17" s="13" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="B19" s="5"/>
+    </row>
+    <row r="20" spans="1:2" ht="52.8" x14ac:dyDescent="0.25">
+      <c r="A20" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="B20" s="13" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="B21" s="13" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="B22" s="13" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="B23" s="13" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="B24" s="15">
+        <v>46324</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="B25" s="13"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1468,20 +1524,20 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:C17"/>
-  <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:C25"/>
+  <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="24.796875" customWidth="1"/>
-    <col min="2" max="2" width="56.796875" customWidth="1"/>
+    <col min="1" max="1" width="24.77734375" customWidth="1"/>
+    <col min="2" max="2" width="56.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="13.15" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>65</v>
       </c>
       <c r="B1" s="2"/>
     </row>
-    <row r="2" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="10" t="s">
         <v>3</v>
       </c>
@@ -1489,7 +1545,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="44.55" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:3" ht="44.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="10" t="s">
         <v>66</v>
       </c>
@@ -1497,7 +1553,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="125.55" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:3" ht="125.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="10" t="s">
         <v>67</v>
       </c>
@@ -1505,7 +1561,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="112.05" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:3" ht="112.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="10" t="s">
         <v>69</v>
       </c>
@@ -1513,7 +1569,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="58.05" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:3" ht="58.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="10" t="s">
         <v>71</v>
       </c>
@@ -1521,7 +1577,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="193.05" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:3" ht="193.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="10" t="s">
         <v>73</v>
       </c>
@@ -1529,7 +1585,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="10" t="s">
         <v>75</v>
       </c>
@@ -1537,7 +1593,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="12.75" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A9" s="10" t="s">
         <v>77</v>
       </c>
@@ -1545,15 +1601,15 @@
         <v>46323</v>
       </c>
     </row>
-    <row r="10" spans="1:3" ht="12.75" x14ac:dyDescent="0.35"/>
-    <row r="11" spans="1:3" ht="13.15" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:3" ht="13.2" x14ac:dyDescent="0.25"/>
+    <row r="11" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
         <v>65</v>
       </c>
       <c r="B11" s="5"/>
       <c r="C11" s="6"/>
     </row>
-    <row r="12" spans="1:3" ht="179.55" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:3" ht="179.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
         <v>78</v>
       </c>
@@ -1561,7 +1617,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="13" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
         <v>80</v>
       </c>
@@ -1569,7 +1625,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="14" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
         <v>82</v>
       </c>
@@ -1577,7 +1633,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="15" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
         <v>84</v>
       </c>
@@ -1585,7 +1641,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="16" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
         <v>85</v>
       </c>
@@ -1593,15 +1649,65 @@
         <v>46323</v>
       </c>
     </row>
-    <row r="17" spans="1:2" ht="17.55" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:2" ht="17.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
         <v>86</v>
       </c>
-      <c r="B17" s="13" t="inlineStr">
-        <is>
-          <t>70a12f9</t>
-        </is>
-      </c>
+      <c r="B17" s="13" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="B19" s="5"/>
+    </row>
+    <row r="20" spans="1:2" ht="145.19999999999999" x14ac:dyDescent="0.25">
+      <c r="A20" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="B20" s="13" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="B21" s="13" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="B22" s="13" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="B23" s="13" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="B24" s="15">
+        <v>46324</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="B25" s="13"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1613,20 +1719,20 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:C17"/>
-  <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:C25"/>
+  <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="24.796875" customWidth="1"/>
-    <col min="2" max="2" width="56.796875" customWidth="1"/>
+    <col min="1" max="1" width="24.77734375" customWidth="1"/>
+    <col min="2" max="2" width="56.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="13.15" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>65</v>
       </c>
       <c r="B1" s="2"/>
     </row>
-    <row r="2" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="10" t="s">
         <v>3</v>
       </c>
@@ -1634,7 +1740,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="44.55" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:3" ht="44.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="10" t="s">
         <v>66</v>
       </c>
@@ -1642,7 +1748,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="71.55" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:3" ht="71.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="10" t="s">
         <v>67</v>
       </c>
@@ -1650,7 +1756,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="31.05" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:3" ht="31.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="10" t="s">
         <v>69</v>
       </c>
@@ -1658,7 +1764,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="31.05" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:3" ht="31.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="10" t="s">
         <v>71</v>
       </c>
@@ -1666,7 +1772,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="71.55" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:3" ht="71.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="10" t="s">
         <v>73</v>
       </c>
@@ -1674,7 +1780,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="10" t="s">
         <v>75</v>
       </c>
@@ -1682,7 +1788,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="12.75" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A9" s="10" t="s">
         <v>77</v>
       </c>
@@ -1690,15 +1796,15 @@
         <v>46323</v>
       </c>
     </row>
-    <row r="10" spans="1:3" ht="12.75" x14ac:dyDescent="0.35"/>
-    <row r="11" spans="1:3" ht="13.15" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:3" ht="13.2" x14ac:dyDescent="0.25"/>
+    <row r="11" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
         <v>65</v>
       </c>
       <c r="B11" s="5"/>
       <c r="C11" s="6"/>
     </row>
-    <row r="12" spans="1:3" ht="71.55" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:3" ht="71.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
         <v>78</v>
       </c>
@@ -1706,7 +1812,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="13" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
         <v>80</v>
       </c>
@@ -1714,7 +1820,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="14" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
         <v>82</v>
       </c>
@@ -1722,7 +1828,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="15" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
         <v>84</v>
       </c>
@@ -1730,7 +1836,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="16" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
         <v>85</v>
       </c>
@@ -1738,15 +1844,65 @@
         <v>46323</v>
       </c>
     </row>
-    <row r="17" spans="1:2" ht="17.55" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:2" ht="17.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
         <v>86</v>
       </c>
-      <c r="B17" s="13" t="inlineStr">
-        <is>
-          <t>70a12f9</t>
-        </is>
-      </c>
+      <c r="B17" s="13" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="B19" s="5"/>
+    </row>
+    <row r="20" spans="1:2" ht="52.8" x14ac:dyDescent="0.25">
+      <c r="A20" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="B20" s="13" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="B21" s="13" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="B22" s="13" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="B23" s="13" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="B24" s="15">
+        <v>46324</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="B25" s="13"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1758,20 +1914,20 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:C17"/>
-  <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:C25"/>
+  <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="24.796875" customWidth="1"/>
-    <col min="2" max="2" width="56.796875" customWidth="1"/>
+    <col min="1" max="1" width="24.77734375" customWidth="1"/>
+    <col min="2" max="2" width="56.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="13.15" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>65</v>
       </c>
       <c r="B1" s="2"/>
     </row>
-    <row r="2" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="10" t="s">
         <v>3</v>
       </c>
@@ -1779,7 +1935,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="31.05" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:3" ht="31.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="10" t="s">
         <v>66</v>
       </c>
@@ -1787,7 +1943,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="85.05" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:3" ht="85.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="10" t="s">
         <v>67</v>
       </c>
@@ -1795,7 +1951,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="85.05" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:3" ht="85.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="10" t="s">
         <v>69</v>
       </c>
@@ -1803,7 +1959,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="31.05" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:3" ht="31.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="10" t="s">
         <v>71</v>
       </c>
@@ -1811,7 +1967,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="98.55" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:3" ht="98.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="10" t="s">
         <v>73</v>
       </c>
@@ -1819,7 +1975,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="10" t="s">
         <v>75</v>
       </c>
@@ -1827,7 +1983,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="12.75" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A9" s="10" t="s">
         <v>77</v>
       </c>
@@ -1835,15 +1991,15 @@
         <v>46323</v>
       </c>
     </row>
-    <row r="10" spans="1:3" ht="12.75" x14ac:dyDescent="0.35"/>
-    <row r="11" spans="1:3" ht="13.15" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:3" ht="13.2" x14ac:dyDescent="0.25"/>
+    <row r="11" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
         <v>65</v>
       </c>
       <c r="B11" s="5"/>
       <c r="C11" s="6"/>
     </row>
-    <row r="12" spans="1:3" ht="85.05" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:3" ht="85.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
         <v>78</v>
       </c>
@@ -1851,7 +2007,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="13" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
         <v>80</v>
       </c>
@@ -1859,7 +2015,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="14" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
         <v>82</v>
       </c>
@@ -1867,7 +2023,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="15" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
         <v>84</v>
       </c>
@@ -1875,7 +2031,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="16" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
         <v>85</v>
       </c>
@@ -1883,15 +2039,65 @@
         <v>46323</v>
       </c>
     </row>
-    <row r="17" spans="1:2" ht="17.55" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:2" ht="17.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
         <v>86</v>
       </c>
-      <c r="B17" s="13" t="inlineStr">
-        <is>
-          <t>70a12f9</t>
-        </is>
-      </c>
+      <c r="B17" s="13" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="B19" s="5"/>
+    </row>
+    <row r="20" spans="1:2" ht="66" x14ac:dyDescent="0.25">
+      <c r="A20" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="B20" s="13" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="B21" s="13" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="B22" s="13" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="B23" s="13" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="B24" s="15">
+        <v>46324</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="B25" s="13"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1903,20 +2109,20 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:C17"/>
-  <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:C25"/>
+  <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="24.796875" customWidth="1"/>
-    <col min="2" max="2" width="56.796875" customWidth="1"/>
+    <col min="1" max="1" width="24.77734375" customWidth="1"/>
+    <col min="2" max="2" width="56.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="13.15" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>65</v>
       </c>
       <c r="B1" s="2"/>
     </row>
-    <row r="2" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="10" t="s">
         <v>3</v>
       </c>
@@ -1924,7 +2130,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="31.05" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:3" ht="31.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="10" t="s">
         <v>66</v>
       </c>
@@ -1932,7 +2138,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="58.05" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:3" ht="58.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="10" t="s">
         <v>67</v>
       </c>
@@ -1940,7 +2146,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="166.05" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:3" ht="166.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="10" t="s">
         <v>69</v>
       </c>
@@ -1948,7 +2154,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="44.55" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:3" ht="44.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="10" t="s">
         <v>71</v>
       </c>
@@ -1956,7 +2162,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="166.05" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:3" ht="166.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="10" t="s">
         <v>73</v>
       </c>
@@ -1964,7 +2170,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="10" t="s">
         <v>75</v>
       </c>
@@ -1972,7 +2178,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="12.75" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A9" s="10" t="s">
         <v>77</v>
       </c>
@@ -1980,15 +2186,15 @@
         <v>46323</v>
       </c>
     </row>
-    <row r="10" spans="1:3" ht="12.75" x14ac:dyDescent="0.35"/>
-    <row r="11" spans="1:3" ht="13.15" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:3" ht="13.2" x14ac:dyDescent="0.25"/>
+    <row r="11" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
         <v>65</v>
       </c>
       <c r="B11" s="5"/>
       <c r="C11" s="6"/>
     </row>
-    <row r="12" spans="1:3" ht="112.05" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:3" ht="112.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
         <v>78</v>
       </c>
@@ -1996,7 +2202,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="13" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
         <v>80</v>
       </c>
@@ -2004,7 +2210,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="14" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
         <v>82</v>
       </c>
@@ -2012,7 +2218,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="15" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
         <v>84</v>
       </c>
@@ -2020,7 +2226,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="16" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
         <v>85</v>
       </c>
@@ -2028,15 +2234,65 @@
         <v>46323</v>
       </c>
     </row>
-    <row r="17" spans="1:2" ht="17.55" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:2" ht="17.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
         <v>86</v>
       </c>
-      <c r="B17" s="13" t="inlineStr">
-        <is>
-          <t>70a12f9</t>
-        </is>
-      </c>
+      <c r="B17" s="13" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="B19" s="5"/>
+    </row>
+    <row r="20" spans="1:2" ht="92.4" x14ac:dyDescent="0.25">
+      <c r="A20" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="B20" s="13" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="B21" s="13" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="B22" s="13" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="B23" s="13" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="B24" s="15">
+        <v>46324</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="B25" s="13"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2048,20 +2304,20 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:C17"/>
-  <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:C25"/>
+  <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="24.796875" customWidth="1"/>
-    <col min="2" max="2" width="56.796875" customWidth="1"/>
+    <col min="1" max="1" width="24.77734375" customWidth="1"/>
+    <col min="2" max="2" width="56.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="13.15" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>65</v>
       </c>
       <c r="B1" s="2"/>
     </row>
-    <row r="2" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="10" t="s">
         <v>3</v>
       </c>
@@ -2069,7 +2325,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="31.05" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:3" ht="31.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="10" t="s">
         <v>66</v>
       </c>
@@ -2077,7 +2333,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="85.05" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:3" ht="85.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="10" t="s">
         <v>67</v>
       </c>
@@ -2085,7 +2341,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="112.05" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:3" ht="112.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="10" t="s">
         <v>69</v>
       </c>
@@ -2093,7 +2349,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="31.05" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:3" ht="31.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="10" t="s">
         <v>71</v>
       </c>
@@ -2101,7 +2357,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="85.05" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:3" ht="85.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="10" t="s">
         <v>73</v>
       </c>
@@ -2109,7 +2365,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="10" t="s">
         <v>75</v>
       </c>
@@ -2117,7 +2373,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="12.75" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A9" s="10" t="s">
         <v>77</v>
       </c>
@@ -2125,15 +2381,15 @@
         <v>46323</v>
       </c>
     </row>
-    <row r="10" spans="1:3" ht="12.75" x14ac:dyDescent="0.35"/>
-    <row r="11" spans="1:3" ht="13.15" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:3" ht="13.2" x14ac:dyDescent="0.25"/>
+    <row r="11" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
         <v>65</v>
       </c>
       <c r="B11" s="5"/>
       <c r="C11" s="6"/>
     </row>
-    <row r="12" spans="1:3" ht="58.05" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:3" ht="58.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
         <v>78</v>
       </c>
@@ -2141,7 +2397,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="13" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
         <v>80</v>
       </c>
@@ -2149,7 +2405,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="14" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
         <v>82</v>
       </c>
@@ -2157,7 +2413,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="15" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
         <v>84</v>
       </c>
@@ -2165,7 +2421,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="16" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
         <v>85</v>
       </c>
@@ -2173,15 +2429,65 @@
         <v>46323</v>
       </c>
     </row>
-    <row r="17" spans="1:2" ht="17.55" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:2" ht="17.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
         <v>86</v>
       </c>
-      <c r="B17" s="13" t="inlineStr">
-        <is>
-          <t>70a12f9</t>
-        </is>
-      </c>
+      <c r="B17" s="13" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="B19" s="5"/>
+    </row>
+    <row r="20" spans="1:2" ht="52.8" x14ac:dyDescent="0.25">
+      <c r="A20" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="B20" s="13" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="B21" s="13" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="B22" s="13" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="B23" s="13" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="B24" s="15">
+        <v>46324</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="B25" s="13"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2193,20 +2499,20 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:C17"/>
-  <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:C25"/>
+  <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="24.796875" customWidth="1"/>
-    <col min="2" max="2" width="56.796875" customWidth="1"/>
+    <col min="1" max="1" width="24.77734375" customWidth="1"/>
+    <col min="2" max="2" width="56.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="13.15" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>65</v>
       </c>
       <c r="B1" s="2"/>
     </row>
-    <row r="2" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="10" t="s">
         <v>3</v>
       </c>
@@ -2214,7 +2520,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="44.55" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:3" ht="44.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="10" t="s">
         <v>66</v>
       </c>
@@ -2222,7 +2528,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="112.05" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:3" ht="112.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="10" t="s">
         <v>67</v>
       </c>
@@ -2230,7 +2536,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="44.55" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:3" ht="44.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="10" t="s">
         <v>69</v>
       </c>
@@ -2238,7 +2544,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="31.05" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:3" ht="31.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="10" t="s">
         <v>71</v>
       </c>
@@ -2246,7 +2552,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="98.55" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:3" ht="98.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="10" t="s">
         <v>73</v>
       </c>
@@ -2254,7 +2560,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="10" t="s">
         <v>75</v>
       </c>
@@ -2262,7 +2568,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="12.75" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A9" s="10" t="s">
         <v>77</v>
       </c>
@@ -2270,15 +2576,15 @@
         <v>46323</v>
       </c>
     </row>
-    <row r="10" spans="1:3" ht="12.75" x14ac:dyDescent="0.35"/>
-    <row r="11" spans="1:3" ht="13.15" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:3" ht="13.2" x14ac:dyDescent="0.25"/>
+    <row r="11" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
         <v>65</v>
       </c>
       <c r="B11" s="5"/>
       <c r="C11" s="6"/>
     </row>
-    <row r="12" spans="1:3" ht="98.55" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:3" ht="98.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
         <v>78</v>
       </c>
@@ -2286,7 +2592,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="13" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
         <v>80</v>
       </c>
@@ -2294,7 +2600,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="14" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
         <v>82</v>
       </c>
@@ -2302,7 +2608,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="15" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
         <v>84</v>
       </c>
@@ -2310,7 +2616,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="16" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
         <v>85</v>
       </c>
@@ -2318,15 +2624,65 @@
         <v>46323</v>
       </c>
     </row>
-    <row r="17" spans="1:2" ht="17.55" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:2" ht="17.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
         <v>86</v>
       </c>
-      <c r="B17" s="13" t="inlineStr">
-        <is>
-          <t>70a12f9</t>
-        </is>
-      </c>
+      <c r="B17" s="13" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="B19" s="5"/>
+    </row>
+    <row r="20" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="B20" s="13" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="B21" s="13" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="B22" s="13" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="B23" s="13" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="B24" s="15">
+        <v>46324</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="B25" s="13"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2338,20 +2694,20 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:C17"/>
-  <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:C25"/>
+  <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="24.796875" customWidth="1"/>
-    <col min="2" max="2" width="56.796875" customWidth="1"/>
+    <col min="1" max="1" width="24.77734375" customWidth="1"/>
+    <col min="2" max="2" width="56.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="13.15" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>65</v>
       </c>
       <c r="B1" s="2"/>
     </row>
-    <row r="2" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="10" t="s">
         <v>3</v>
       </c>
@@ -2359,7 +2715,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="31.05" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:3" ht="31.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="10" t="s">
         <v>66</v>
       </c>
@@ -2367,7 +2723,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="125.55" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:3" ht="125.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="10" t="s">
         <v>67</v>
       </c>
@@ -2375,7 +2731,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="125.55" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:3" ht="125.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="10" t="s">
         <v>69</v>
       </c>
@@ -2383,7 +2739,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="44.55" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:3" ht="44.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="10" t="s">
         <v>71</v>
       </c>
@@ -2391,7 +2747,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="166.05" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:3" ht="166.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="10" t="s">
         <v>73</v>
       </c>
@@ -2399,7 +2755,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="10" t="s">
         <v>75</v>
       </c>
@@ -2407,7 +2763,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="12.75" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A9" s="10" t="s">
         <v>77</v>
       </c>
@@ -2415,15 +2771,15 @@
         <v>46323</v>
       </c>
     </row>
-    <row r="10" spans="1:3" ht="12.75" x14ac:dyDescent="0.35"/>
-    <row r="11" spans="1:3" ht="13.15" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:3" ht="13.2" x14ac:dyDescent="0.25"/>
+    <row r="11" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
         <v>65</v>
       </c>
       <c r="B11" s="5"/>
       <c r="C11" s="6"/>
     </row>
-    <row r="12" spans="1:3" ht="139.05000000000001" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:3" ht="139.05000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
         <v>78</v>
       </c>
@@ -2431,7 +2787,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="13" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
         <v>80</v>
       </c>
@@ -2439,7 +2795,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="14" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
         <v>82</v>
       </c>
@@ -2447,7 +2803,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="15" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
         <v>84</v>
       </c>
@@ -2455,7 +2811,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="16" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
         <v>85</v>
       </c>
@@ -2463,15 +2819,65 @@
         <v>46323</v>
       </c>
     </row>
-    <row r="17" spans="1:2" ht="17.55" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:2" ht="17.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
         <v>86</v>
       </c>
-      <c r="B17" s="13" t="inlineStr">
-        <is>
-          <t>70a12f9</t>
-        </is>
-      </c>
+      <c r="B17" s="13" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="B19" s="5"/>
+    </row>
+    <row r="20" spans="1:2" ht="118.8" x14ac:dyDescent="0.25">
+      <c r="A20" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="B20" s="13" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="B21" s="13" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="B22" s="13" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="B23" s="13" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="B24" s="15">
+        <v>46324</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="B25" s="13"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2483,20 +2889,20 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:C17"/>
-  <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:C25"/>
+  <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="24.796875" customWidth="1"/>
-    <col min="2" max="2" width="56.796875" customWidth="1"/>
+    <col min="1" max="1" width="24.77734375" customWidth="1"/>
+    <col min="2" max="2" width="56.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="13.15" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>65</v>
       </c>
       <c r="B1" s="2"/>
     </row>
-    <row r="2" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="10" t="s">
         <v>3</v>
       </c>
@@ -2504,7 +2910,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="31.05" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:3" ht="31.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="10" t="s">
         <v>66</v>
       </c>
@@ -2512,7 +2918,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="98.55" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:3" ht="98.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="10" t="s">
         <v>67</v>
       </c>
@@ -2520,7 +2926,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="85.05" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:3" ht="85.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="10" t="s">
         <v>69</v>
       </c>
@@ -2528,7 +2934,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="31.05" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:3" ht="31.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="10" t="s">
         <v>71</v>
       </c>
@@ -2536,7 +2942,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="58.05" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:3" ht="58.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="10" t="s">
         <v>73</v>
       </c>
@@ -2544,7 +2950,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="10" t="s">
         <v>75</v>
       </c>
@@ -2552,7 +2958,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="12.75" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A9" s="10" t="s">
         <v>77</v>
       </c>
@@ -2560,15 +2966,15 @@
         <v>46323</v>
       </c>
     </row>
-    <row r="10" spans="1:3" ht="12.75" x14ac:dyDescent="0.35"/>
-    <row r="11" spans="1:3" ht="13.15" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:3" ht="13.2" x14ac:dyDescent="0.25"/>
+    <row r="11" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
         <v>65</v>
       </c>
       <c r="B11" s="5"/>
       <c r="C11" s="6"/>
     </row>
-    <row r="12" spans="1:3" ht="71.55" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:3" ht="71.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
         <v>78</v>
       </c>
@@ -2576,7 +2982,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="13" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
         <v>80</v>
       </c>
@@ -2584,7 +2990,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="14" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
         <v>82</v>
       </c>
@@ -2592,7 +2998,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="15" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
         <v>84</v>
       </c>
@@ -2600,7 +3006,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="16" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
         <v>85</v>
       </c>
@@ -2608,15 +3014,65 @@
         <v>46323</v>
       </c>
     </row>
-    <row r="17" spans="1:2" ht="17.55" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:2" ht="17.55" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
         <v>86</v>
       </c>
-      <c r="B17" s="13" t="inlineStr">
-        <is>
-          <t>70a12f9</t>
-        </is>
-      </c>
+      <c r="B17" s="13" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="B19" s="5"/>
+    </row>
+    <row r="20" spans="1:2" ht="66" x14ac:dyDescent="0.25">
+      <c r="A20" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="B20" s="13" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="B21" s="13" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="B22" s="13" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="B23" s="13" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="B24" s="15">
+        <v>46324</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="B25" s="13"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
SPM-57: Fill in the Commit cells for Kristen's test case run
The pre-commit hook couldn't write them in a13e6fa because the workbook
was open in Excel. 95672dd is the build that was tested.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/test-cases/SPM-57_Test_Cases.xlsx
+++ b/docs/test-cases/SPM-57_Test_Cases.xlsx
@@ -1512,7 +1512,11 @@
       <c r="A25" s="3" t="s">
         <v>86</v>
       </c>
-      <c r="B25" s="13"/>
+      <c r="B25" s="13" t="inlineStr">
+        <is>
+          <t>95672dd</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1707,7 +1711,11 @@
       <c r="A25" s="3" t="s">
         <v>86</v>
       </c>
-      <c r="B25" s="13"/>
+      <c r="B25" s="13" t="inlineStr">
+        <is>
+          <t>95672dd</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1902,7 +1910,11 @@
       <c r="A25" s="3" t="s">
         <v>86</v>
       </c>
-      <c r="B25" s="13"/>
+      <c r="B25" s="13" t="inlineStr">
+        <is>
+          <t>95672dd</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2097,7 +2109,11 @@
       <c r="A25" s="3" t="s">
         <v>86</v>
       </c>
-      <c r="B25" s="13"/>
+      <c r="B25" s="13" t="inlineStr">
+        <is>
+          <t>95672dd</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2292,7 +2308,11 @@
       <c r="A25" s="3" t="s">
         <v>86</v>
       </c>
-      <c r="B25" s="13"/>
+      <c r="B25" s="13" t="inlineStr">
+        <is>
+          <t>95672dd</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2487,7 +2507,11 @@
       <c r="A25" s="3" t="s">
         <v>86</v>
       </c>
-      <c r="B25" s="13"/>
+      <c r="B25" s="13" t="inlineStr">
+        <is>
+          <t>95672dd</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2682,7 +2706,11 @@
       <c r="A25" s="3" t="s">
         <v>86</v>
       </c>
-      <c r="B25" s="13"/>
+      <c r="B25" s="13" t="inlineStr">
+        <is>
+          <t>95672dd</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2877,7 +2905,11 @@
       <c r="A25" s="3" t="s">
         <v>86</v>
       </c>
-      <c r="B25" s="13"/>
+      <c r="B25" s="13" t="inlineStr">
+        <is>
+          <t>95672dd</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3072,7 +3104,11 @@
       <c r="A25" s="3" t="s">
         <v>86</v>
       </c>
-      <c r="B25" s="13"/>
+      <c r="B25" s="13" t="inlineStr">
+        <is>
+          <t>95672dd</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>